<commit_message>
Intégration de la gestion des badges des élèves dans le dashboard.html, le base.html et les autres templates de liste
</commit_message>
<xml_diff>
--- a/imports/Classe.xlsx
+++ b/imports/Classe.xlsx
@@ -9,6 +9,7 @@
     <sheet name="A" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">A!$A$1:$I$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">A!$A$1:$I$15</definedName>
   </definedNames>
   <calcPr/>
@@ -196,7 +197,7 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
       <protection locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" applyProtection="0">
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="1"/>
     </xf>
@@ -729,7 +730,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" ht="13.5" customHeight="1">
+    <row r="3" ht="13.5" hidden="1" customHeight="1">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -758,7 +759,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" ht="13.5" customHeight="1">
+    <row r="4" ht="13.5" hidden="1" customHeight="1">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -787,7 +788,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" ht="13.5" customHeight="1">
+    <row r="5" ht="13.5" hidden="1" customHeight="1">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -845,7 +846,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" ht="13.5" hidden="1" customHeight="1">
+    <row r="7" ht="13.5" customHeight="1">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -1110,9 +1111,7 @@
   <autoFilter ref="A1:I15">
     <filterColumn colId="8">
       <filters>
-        <filter val="MATEM7"/>
-        <filter val="MATEP6"/>
-        <filter val="MATET5"/>
+        <filter val="PRIMC9"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>